<commit_message>
fix: data URL 不被 base_url 覆盖，smoke 用例改用 base64 编码
</commit_message>
<xml_diff>
--- a/projects/demo/smoke_cases.xlsx
+++ b/projects/demo/smoke_cases.xlsx
@@ -472,7 +472,11 @@
           <t>go</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>data:text/html;base64,PGgxPldlYlRlc3QgT0s8L2gxPjxwPlBpcGVsaW5lIHdvcmtzPC9wPg==</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>data:text/html,&lt;h1&gt;WebTest OK&lt;/h1&gt;&lt;p&gt;Pipeline works&lt;/p&gt;</t>
@@ -503,7 +507,6 @@
           <t>assert_text</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>WebTest OK</t>

</xml_diff>